<commit_message>
Regenerate sample company XLSX with less volatile financial data
Smoothed the SampleCompanyData.xlsx spreadsheet directly using outlier
capping (2.5x product median) and two-pass moving average (5-month then
3-month). Revenue monthly totals now range ~$10.5k-$17k (was $5.9k-$23.2k)
and expenses ~$5.7k-$14.5k (was $4k-$25.3k).

Removed the runtime SmoothMonthlyTransactions code from SampleCompanyService
since smoothing is now baked into the spreadsheet data itself.

Added a RegenerateSampleData tool (skipped xUnit test) for future XLSX
regeneration.

https://claude.ai/code/session_01DPg7EhwGYWg5XCpB2GBKvu
</commit_message>
<xml_diff>
--- a/ArgoBooks/Resources/SampleCompanyData.xlsx
+++ b/ArgoBooks/Resources/SampleCompanyData.xlsx
@@ -1571,13 +1571,13 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1299</v>
+        <v>1189.03</v>
       </c>
       <c r="F2" t="n">
-        <v>107.17</v>
+        <v>98.09999999999999</v>
       </c>
       <c r="G2" t="n">
-        <v>1406.17</v>
+        <v>1287.12</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -1615,13 +1615,13 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>1299</v>
+        <v>1189.03</v>
       </c>
       <c r="F3" t="n">
-        <v>107.17</v>
+        <v>98.09999999999999</v>
       </c>
       <c r="G3" t="n">
-        <v>1406.17</v>
+        <v>1287.12</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -1659,13 +1659,13 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>1299</v>
+        <v>1189.03</v>
       </c>
       <c r="F4" t="n">
-        <v>107.17</v>
+        <v>98.09999999999999</v>
       </c>
       <c r="G4" t="n">
-        <v>1406.17</v>
+        <v>1287.12</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -1700,13 +1700,13 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>549</v>
+        <v>502.52</v>
       </c>
       <c r="F5" t="n">
-        <v>45.29</v>
+        <v>41.46</v>
       </c>
       <c r="G5" t="n">
-        <v>594.29</v>
+        <v>543.98</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -1744,13 +1744,13 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>549</v>
+        <v>502.52</v>
       </c>
       <c r="F6" t="n">
-        <v>45.29</v>
+        <v>41.46</v>
       </c>
       <c r="G6" t="n">
-        <v>594.29</v>
+        <v>543.98</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -1785,13 +1785,13 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>899</v>
+        <v>822.89</v>
       </c>
       <c r="F7" t="n">
-        <v>74.17</v>
+        <v>67.89</v>
       </c>
       <c r="G7" t="n">
-        <v>973.17</v>
+        <v>890.78</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -1826,13 +1826,13 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>899</v>
+        <v>822.89</v>
       </c>
       <c r="F8" t="n">
-        <v>74.17</v>
+        <v>67.89</v>
       </c>
       <c r="G8" t="n">
-        <v>973.17</v>
+        <v>890.78</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -1867,13 +1867,13 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>899</v>
+        <v>822.89</v>
       </c>
       <c r="F9" t="n">
-        <v>74.17</v>
+        <v>67.89</v>
       </c>
       <c r="G9" t="n">
-        <v>973.17</v>
+        <v>890.78</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -1911,13 +1911,13 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>899</v>
+        <v>822.89</v>
       </c>
       <c r="F10" t="n">
-        <v>74.17</v>
+        <v>67.89</v>
       </c>
       <c r="G10" t="n">
-        <v>973.17</v>
+        <v>890.78</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -1955,13 +1955,13 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>249</v>
+        <v>227.92</v>
       </c>
       <c r="F11" t="n">
-        <v>20.54</v>
+        <v>18.8</v>
       </c>
       <c r="G11" t="n">
-        <v>269.54</v>
+        <v>246.72</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -1999,13 +1999,13 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>249</v>
+        <v>227.92</v>
       </c>
       <c r="F12" t="n">
-        <v>20.54</v>
+        <v>18.8</v>
       </c>
       <c r="G12" t="n">
-        <v>269.54</v>
+        <v>246.72</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -2043,13 +2043,13 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>1200</v>
+        <v>1291.7</v>
       </c>
       <c r="F13" t="n">
-        <v>99</v>
+        <v>106.57</v>
       </c>
       <c r="G13" t="n">
-        <v>1299</v>
+        <v>1398.27</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -2087,13 +2087,13 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>1149</v>
+        <v>1236.8</v>
       </c>
       <c r="F14" t="n">
-        <v>94.79000000000001</v>
+        <v>102.03</v>
       </c>
       <c r="G14" t="n">
-        <v>1243.79</v>
+        <v>1338.84</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -2131,13 +2131,13 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>1149</v>
+        <v>1236.8</v>
       </c>
       <c r="F15" t="n">
-        <v>94.79000000000001</v>
+        <v>102.03</v>
       </c>
       <c r="G15" t="n">
-        <v>1243.79</v>
+        <v>1338.84</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -2175,13 +2175,13 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>1149</v>
+        <v>1236.8</v>
       </c>
       <c r="F16" t="n">
-        <v>94.79000000000001</v>
+        <v>102.03</v>
       </c>
       <c r="G16" t="n">
-        <v>1243.79</v>
+        <v>1338.84</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -2219,13 +2219,13 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>1895</v>
+        <v>2039.81</v>
       </c>
       <c r="F17" t="n">
-        <v>156.34</v>
+        <v>168.29</v>
       </c>
       <c r="G17" t="n">
-        <v>2051.34</v>
+        <v>2208.1</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -2260,13 +2260,13 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>1200</v>
+        <v>1215.14</v>
       </c>
       <c r="F18" t="n">
-        <v>99</v>
+        <v>100.25</v>
       </c>
       <c r="G18" t="n">
-        <v>1299</v>
+        <v>1315.39</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -2304,13 +2304,13 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>1299</v>
+        <v>1315.39</v>
       </c>
       <c r="F19" t="n">
-        <v>107.17</v>
+        <v>108.52</v>
       </c>
       <c r="G19" t="n">
-        <v>1406.17</v>
+        <v>1423.91</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -2345,13 +2345,13 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>1299</v>
+        <v>1315.39</v>
       </c>
       <c r="F20" t="n">
-        <v>107.17</v>
+        <v>108.52</v>
       </c>
       <c r="G20" t="n">
-        <v>1406.17</v>
+        <v>1423.91</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -2386,13 +2386,13 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>249</v>
+        <v>252.14</v>
       </c>
       <c r="F21" t="n">
-        <v>20.54</v>
+        <v>20.8</v>
       </c>
       <c r="G21" t="n">
-        <v>269.54</v>
+        <v>272.94</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -2430,13 +2430,13 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>899</v>
+        <v>910.34</v>
       </c>
       <c r="F22" t="n">
-        <v>74.17</v>
+        <v>75.11</v>
       </c>
       <c r="G22" t="n">
-        <v>973.17</v>
+        <v>985.45</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -2471,13 +2471,13 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>899</v>
+        <v>910.34</v>
       </c>
       <c r="F23" t="n">
-        <v>74.17</v>
+        <v>75.11</v>
       </c>
       <c r="G23" t="n">
-        <v>973.17</v>
+        <v>985.45</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -2515,13 +2515,13 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>249</v>
+        <v>252.14</v>
       </c>
       <c r="F24" t="n">
-        <v>20.54</v>
+        <v>20.8</v>
       </c>
       <c r="G24" t="n">
-        <v>269.54</v>
+        <v>272.94</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
@@ -2559,13 +2559,13 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>1200</v>
+        <v>1327.5</v>
       </c>
       <c r="F25" t="n">
-        <v>99</v>
+        <v>109.52</v>
       </c>
       <c r="G25" t="n">
-        <v>1299</v>
+        <v>1437.02</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
@@ -2603,13 +2603,13 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>2899</v>
+        <v>3207.03</v>
       </c>
       <c r="F26" t="n">
-        <v>239.17</v>
+        <v>264.58</v>
       </c>
       <c r="G26" t="n">
-        <v>3138.17</v>
+        <v>3471.61</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
@@ -2647,13 +2647,13 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>2899</v>
+        <v>3207.03</v>
       </c>
       <c r="F27" t="n">
-        <v>239.17</v>
+        <v>264.58</v>
       </c>
       <c r="G27" t="n">
-        <v>3138.17</v>
+        <v>3471.61</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
@@ -2688,13 +2688,13 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>549</v>
+        <v>607.33</v>
       </c>
       <c r="F28" t="n">
-        <v>45.29</v>
+        <v>50.1</v>
       </c>
       <c r="G28" t="n">
-        <v>594.29</v>
+        <v>657.4299999999999</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
@@ -2732,13 +2732,13 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>549</v>
+        <v>607.33</v>
       </c>
       <c r="F29" t="n">
-        <v>45.29</v>
+        <v>50.1</v>
       </c>
       <c r="G29" t="n">
-        <v>594.29</v>
+        <v>657.4299999999999</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
@@ -2773,13 +2773,13 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>1299</v>
+        <v>1437.02</v>
       </c>
       <c r="F30" t="n">
-        <v>107.17</v>
+        <v>118.56</v>
       </c>
       <c r="G30" t="n">
-        <v>1406.17</v>
+        <v>1555.58</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
@@ -2817,13 +2817,13 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>1299</v>
+        <v>1437.02</v>
       </c>
       <c r="F31" t="n">
-        <v>107.17</v>
+        <v>118.56</v>
       </c>
       <c r="G31" t="n">
-        <v>1406.17</v>
+        <v>1555.58</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
@@ -2861,13 +2861,13 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>1200</v>
+        <v>1119.22</v>
       </c>
       <c r="F32" t="n">
-        <v>99</v>
+        <v>92.34</v>
       </c>
       <c r="G32" t="n">
-        <v>1299</v>
+        <v>1211.56</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
@@ -2905,13 +2905,13 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>1899</v>
+        <v>1771.17</v>
       </c>
       <c r="F33" t="n">
-        <v>156.67</v>
+        <v>146.12</v>
       </c>
       <c r="G33" t="n">
-        <v>2055.67</v>
+        <v>1917.3</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
@@ -2949,13 +2949,13 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>1899</v>
+        <v>1771.17</v>
       </c>
       <c r="F34" t="n">
-        <v>156.67</v>
+        <v>146.12</v>
       </c>
       <c r="G34" t="n">
-        <v>2055.67</v>
+        <v>1917.3</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
@@ -2990,13 +2990,13 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>1899</v>
+        <v>1771.17</v>
       </c>
       <c r="F35" t="n">
-        <v>156.67</v>
+        <v>146.12</v>
       </c>
       <c r="G35" t="n">
-        <v>2055.67</v>
+        <v>1917.3</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
@@ -3034,13 +3034,13 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>2195</v>
+        <v>2047.25</v>
       </c>
       <c r="F36" t="n">
-        <v>181.09</v>
+        <v>168.9</v>
       </c>
       <c r="G36" t="n">
-        <v>2376.09</v>
+        <v>2216.15</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
@@ -3078,13 +3078,13 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>1200</v>
+        <v>890.8200000000001</v>
       </c>
       <c r="F37" t="n">
-        <v>99</v>
+        <v>73.48999999999999</v>
       </c>
       <c r="G37" t="n">
-        <v>1299</v>
+        <v>964.3200000000001</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
@@ -3119,13 +3119,13 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>2899</v>
+        <v>2152.08</v>
       </c>
       <c r="F38" t="n">
-        <v>239.17</v>
+        <v>177.55</v>
       </c>
       <c r="G38" t="n">
-        <v>3138.17</v>
+        <v>2329.63</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
@@ -3160,13 +3160,13 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>2899</v>
+        <v>2152.08</v>
       </c>
       <c r="F39" t="n">
-        <v>239.17</v>
+        <v>177.55</v>
       </c>
       <c r="G39" t="n">
-        <v>3138.17</v>
+        <v>2329.63</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
@@ -3204,13 +3204,13 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>549</v>
+        <v>407.55</v>
       </c>
       <c r="F40" t="n">
-        <v>45.29</v>
+        <v>33.62</v>
       </c>
       <c r="G40" t="n">
-        <v>594.29</v>
+        <v>441.17</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
@@ -3245,13 +3245,13 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>3500</v>
+        <v>2598.24</v>
       </c>
       <c r="F41" t="n">
-        <v>288.75</v>
+        <v>214.35</v>
       </c>
       <c r="G41" t="n">
-        <v>3788.75</v>
+        <v>2812.59</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
@@ -3286,13 +3286,13 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>4200</v>
+        <v>3117.89</v>
       </c>
       <c r="F42" t="n">
-        <v>346.5</v>
+        <v>257.23</v>
       </c>
       <c r="G42" t="n">
-        <v>4546.5</v>
+        <v>3375.11</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
@@ -3327,13 +3327,13 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>1200</v>
+        <v>1539.88</v>
       </c>
       <c r="F43" t="n">
-        <v>99</v>
+        <v>127.04</v>
       </c>
       <c r="G43" t="n">
-        <v>1299</v>
+        <v>1666.92</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
@@ -3371,13 +3371,13 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>1299</v>
+        <v>1666.92</v>
       </c>
       <c r="F44" t="n">
-        <v>107.17</v>
+        <v>137.52</v>
       </c>
       <c r="G44" t="n">
-        <v>1406.17</v>
+        <v>1804.44</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
@@ -3412,13 +3412,13 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>1299</v>
+        <v>1666.92</v>
       </c>
       <c r="F45" t="n">
-        <v>107.17</v>
+        <v>137.52</v>
       </c>
       <c r="G45" t="n">
-        <v>1406.17</v>
+        <v>1804.44</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
@@ -3453,13 +3453,13 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>249</v>
+        <v>319.52</v>
       </c>
       <c r="F46" t="n">
-        <v>20.54</v>
+        <v>26.36</v>
       </c>
       <c r="G46" t="n">
-        <v>269.54</v>
+        <v>345.88</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
@@ -3494,13 +3494,13 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>4200</v>
+        <v>5389.57</v>
       </c>
       <c r="F47" t="n">
-        <v>346.5</v>
+        <v>444.64</v>
       </c>
       <c r="G47" t="n">
-        <v>4546.5</v>
+        <v>5834.21</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
@@ -3535,13 +3535,13 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>1200</v>
+        <v>1152.76</v>
       </c>
       <c r="F48" t="n">
-        <v>99</v>
+        <v>95.09999999999999</v>
       </c>
       <c r="G48" t="n">
-        <v>1299</v>
+        <v>1247.86</v>
       </c>
       <c r="H48" t="inlineStr">
         <is>
@@ -3579,13 +3579,13 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>1299</v>
+        <v>1247.86</v>
       </c>
       <c r="F49" t="n">
-        <v>107.17</v>
+        <v>102.95</v>
       </c>
       <c r="G49" t="n">
-        <v>1406.17</v>
+        <v>1350.81</v>
       </c>
       <c r="H49" t="inlineStr">
         <is>
@@ -3620,13 +3620,13 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>249</v>
+        <v>239.2</v>
       </c>
       <c r="F50" t="n">
-        <v>20.54</v>
+        <v>19.73</v>
       </c>
       <c r="G50" t="n">
-        <v>269.54</v>
+        <v>258.93</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
@@ -3664,13 +3664,13 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>1895</v>
+        <v>1820.39</v>
       </c>
       <c r="F51" t="n">
-        <v>156.34</v>
+        <v>150.18</v>
       </c>
       <c r="G51" t="n">
-        <v>2051.34</v>
+        <v>1970.58</v>
       </c>
       <c r="H51" t="inlineStr">
         <is>
@@ -3708,13 +3708,13 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>1200</v>
+        <v>1414.15</v>
       </c>
       <c r="F52" t="n">
-        <v>99</v>
+        <v>116.67</v>
       </c>
       <c r="G52" t="n">
-        <v>1299</v>
+        <v>1530.82</v>
       </c>
       <c r="H52" t="inlineStr">
         <is>
@@ -3752,13 +3752,13 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>899</v>
+        <v>1059.43</v>
       </c>
       <c r="F53" t="n">
-        <v>74.17</v>
+        <v>87.41</v>
       </c>
       <c r="G53" t="n">
-        <v>973.17</v>
+        <v>1146.84</v>
       </c>
       <c r="H53" t="inlineStr">
         <is>
@@ -3796,13 +3796,13 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>899</v>
+        <v>1059.43</v>
       </c>
       <c r="F54" t="n">
-        <v>74.17</v>
+        <v>87.41</v>
       </c>
       <c r="G54" t="n">
-        <v>973.17</v>
+        <v>1146.84</v>
       </c>
       <c r="H54" t="inlineStr">
         <is>
@@ -3840,13 +3840,13 @@
         </is>
       </c>
       <c r="E55" t="n">
-        <v>528</v>
+        <v>622.23</v>
       </c>
       <c r="F55" t="n">
-        <v>43.56</v>
+        <v>51.33</v>
       </c>
       <c r="G55" t="n">
-        <v>571.5599999999999</v>
+        <v>673.5599999999999</v>
       </c>
       <c r="H55" t="inlineStr">
         <is>
@@ -3884,13 +3884,13 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>528</v>
+        <v>622.23</v>
       </c>
       <c r="F56" t="n">
-        <v>43.56</v>
+        <v>51.33</v>
       </c>
       <c r="G56" t="n">
-        <v>571.5599999999999</v>
+        <v>673.5599999999999</v>
       </c>
       <c r="H56" t="inlineStr">
         <is>
@@ -3928,13 +3928,13 @@
         </is>
       </c>
       <c r="E57" t="n">
-        <v>1200</v>
+        <v>2403.32</v>
       </c>
       <c r="F57" t="n">
-        <v>99</v>
+        <v>198.27</v>
       </c>
       <c r="G57" t="n">
-        <v>1299</v>
+        <v>2601.59</v>
       </c>
       <c r="H57" t="inlineStr">
         <is>
@@ -3969,13 +3969,13 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>1299</v>
+        <v>2601.59</v>
       </c>
       <c r="F58" t="n">
-        <v>107.17</v>
+        <v>214.64</v>
       </c>
       <c r="G58" t="n">
-        <v>1406.17</v>
+        <v>2816.23</v>
       </c>
       <c r="H58" t="inlineStr">
         <is>
@@ -4010,13 +4010,13 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>1299</v>
+        <v>2601.59</v>
       </c>
       <c r="F59" t="n">
-        <v>107.17</v>
+        <v>214.64</v>
       </c>
       <c r="G59" t="n">
-        <v>1406.17</v>
+        <v>2816.23</v>
       </c>
       <c r="H59" t="inlineStr">
         <is>
@@ -4054,13 +4054,13 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>249</v>
+        <v>498.69</v>
       </c>
       <c r="F60" t="n">
-        <v>20.54</v>
+        <v>41.14</v>
       </c>
       <c r="G60" t="n">
-        <v>269.54</v>
+        <v>539.83</v>
       </c>
       <c r="H60" t="inlineStr">
         <is>
@@ -4095,13 +4095,13 @@
         </is>
       </c>
       <c r="E61" t="n">
-        <v>699</v>
+        <v>1399.93</v>
       </c>
       <c r="F61" t="n">
-        <v>57.67</v>
+        <v>115.5</v>
       </c>
       <c r="G61" t="n">
-        <v>756.67</v>
+        <v>1515.43</v>
       </c>
       <c r="H61" t="inlineStr">
         <is>
@@ -4136,13 +4136,13 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>699</v>
+        <v>1399.93</v>
       </c>
       <c r="F62" t="n">
-        <v>57.67</v>
+        <v>115.5</v>
       </c>
       <c r="G62" t="n">
-        <v>756.67</v>
+        <v>1515.43</v>
       </c>
       <c r="H62" t="inlineStr">
         <is>
@@ -4180,13 +4180,13 @@
         </is>
       </c>
       <c r="E63" t="n">
-        <v>1200</v>
+        <v>1242.3</v>
       </c>
       <c r="F63" t="n">
-        <v>99</v>
+        <v>102.49</v>
       </c>
       <c r="G63" t="n">
-        <v>1299</v>
+        <v>1344.79</v>
       </c>
       <c r="H63" t="inlineStr">
         <is>
@@ -4221,13 +4221,13 @@
         </is>
       </c>
       <c r="E64" t="n">
-        <v>899</v>
+        <v>930.6900000000001</v>
       </c>
       <c r="F64" t="n">
-        <v>74.17</v>
+        <v>76.78</v>
       </c>
       <c r="G64" t="n">
-        <v>973.17</v>
+        <v>1007.48</v>
       </c>
       <c r="H64" t="inlineStr">
         <is>
@@ -4265,13 +4265,13 @@
         </is>
       </c>
       <c r="E65" t="n">
-        <v>899</v>
+        <v>930.6900000000001</v>
       </c>
       <c r="F65" t="n">
-        <v>74.17</v>
+        <v>76.78</v>
       </c>
       <c r="G65" t="n">
-        <v>973.17</v>
+        <v>1007.48</v>
       </c>
       <c r="H65" t="inlineStr">
         <is>
@@ -4309,13 +4309,13 @@
         </is>
       </c>
       <c r="E66" t="n">
-        <v>249</v>
+        <v>257.78</v>
       </c>
       <c r="F66" t="n">
-        <v>20.54</v>
+        <v>21.26</v>
       </c>
       <c r="G66" t="n">
-        <v>269.54</v>
+        <v>279.04</v>
       </c>
       <c r="H66" t="inlineStr">
         <is>
@@ -4353,13 +4353,13 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>5500</v>
+        <v>5693.9</v>
       </c>
       <c r="F67" t="n">
-        <v>453.75</v>
+        <v>469.75</v>
       </c>
       <c r="G67" t="n">
-        <v>5953.75</v>
+        <v>6163.64</v>
       </c>
       <c r="H67" t="inlineStr">
         <is>
@@ -4394,13 +4394,13 @@
         </is>
       </c>
       <c r="E68" t="n">
-        <v>1200</v>
+        <v>976.46</v>
       </c>
       <c r="F68" t="n">
-        <v>99</v>
+        <v>80.56</v>
       </c>
       <c r="G68" t="n">
-        <v>1299</v>
+        <v>1057.02</v>
       </c>
       <c r="H68" t="inlineStr">
         <is>
@@ -4438,13 +4438,13 @@
         </is>
       </c>
       <c r="E69" t="n">
-        <v>1899</v>
+        <v>1545.25</v>
       </c>
       <c r="F69" t="n">
-        <v>156.67</v>
+        <v>127.49</v>
       </c>
       <c r="G69" t="n">
-        <v>2055.67</v>
+        <v>1672.74</v>
       </c>
       <c r="H69" t="inlineStr">
         <is>
@@ -4479,13 +4479,13 @@
         </is>
       </c>
       <c r="E70" t="n">
-        <v>1899</v>
+        <v>1545.25</v>
       </c>
       <c r="F70" t="n">
-        <v>156.67</v>
+        <v>127.49</v>
       </c>
       <c r="G70" t="n">
-        <v>2055.67</v>
+        <v>1672.74</v>
       </c>
       <c r="H70" t="inlineStr">
         <is>
@@ -4523,13 +4523,13 @@
         </is>
       </c>
       <c r="E71" t="n">
-        <v>3500</v>
+        <v>2848.01</v>
       </c>
       <c r="F71" t="n">
-        <v>288.75</v>
+        <v>234.96</v>
       </c>
       <c r="G71" t="n">
-        <v>3788.75</v>
+        <v>3082.98</v>
       </c>
       <c r="H71" t="inlineStr">
         <is>
@@ -4564,13 +4564,13 @@
         </is>
       </c>
       <c r="E72" t="n">
-        <v>2899</v>
+        <v>2358.97</v>
       </c>
       <c r="F72" t="n">
-        <v>239.17</v>
+        <v>194.62</v>
       </c>
       <c r="G72" t="n">
-        <v>3138.17</v>
+        <v>2553.59</v>
       </c>
       <c r="H72" t="inlineStr">
         <is>
@@ -4605,13 +4605,13 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>549</v>
+        <v>446.73</v>
       </c>
       <c r="F73" t="n">
-        <v>45.29</v>
+        <v>36.85</v>
       </c>
       <c r="G73" t="n">
-        <v>594.29</v>
+        <v>483.58</v>
       </c>
       <c r="H73" t="inlineStr">
         <is>
@@ -4649,13 +4649,13 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>4200</v>
+        <v>3417.62</v>
       </c>
       <c r="F74" t="n">
-        <v>346.5</v>
+        <v>281.95</v>
       </c>
       <c r="G74" t="n">
-        <v>4546.5</v>
+        <v>3699.57</v>
       </c>
       <c r="H74" t="inlineStr">
         <is>
@@ -4693,13 +4693,13 @@
         </is>
       </c>
       <c r="E75" t="n">
-        <v>3500</v>
+        <v>3203.69</v>
       </c>
       <c r="F75" t="n">
-        <v>288.75</v>
+        <v>264.3</v>
       </c>
       <c r="G75" t="n">
-        <v>3788.75</v>
+        <v>3467.99</v>
       </c>
       <c r="H75" t="inlineStr">
         <is>
@@ -4737,13 +4737,13 @@
         </is>
       </c>
       <c r="E76" t="n">
-        <v>4200</v>
+        <v>4520.95</v>
       </c>
       <c r="F76" t="n">
-        <v>346.5</v>
+        <v>372.98</v>
       </c>
       <c r="G76" t="n">
-        <v>4546.5</v>
+        <v>4893.93</v>
       </c>
       <c r="H76" t="inlineStr">
         <is>
@@ -4781,13 +4781,13 @@
         </is>
       </c>
       <c r="E77" t="n">
-        <v>5500</v>
+        <v>5569.38</v>
       </c>
       <c r="F77" t="n">
-        <v>453.75</v>
+        <v>459.47</v>
       </c>
       <c r="G77" t="n">
-        <v>5953.75</v>
+        <v>6028.85</v>
       </c>
       <c r="H77" t="inlineStr">
         <is>
@@ -4822,13 +4822,13 @@
         </is>
       </c>
       <c r="E78" t="n">
-        <v>3500</v>
+        <v>3264.4</v>
       </c>
       <c r="F78" t="n">
-        <v>288.75</v>
+        <v>269.31</v>
       </c>
       <c r="G78" t="n">
-        <v>3788.75</v>
+        <v>3533.72</v>
       </c>
       <c r="H78" t="inlineStr">
         <is>
@@ -4866,13 +4866,13 @@
         </is>
       </c>
       <c r="E79" t="n">
-        <v>5500</v>
+        <v>5283.46</v>
       </c>
       <c r="F79" t="n">
-        <v>453.75</v>
+        <v>435.89</v>
       </c>
       <c r="G79" t="n">
-        <v>5953.75</v>
+        <v>5719.35</v>
       </c>
       <c r="H79" t="inlineStr">
         <is>
@@ -4907,13 +4907,13 @@
         </is>
       </c>
       <c r="E80" t="n">
-        <v>4200</v>
+        <v>4949.53</v>
       </c>
       <c r="F80" t="n">
-        <v>346.5</v>
+        <v>408.34</v>
       </c>
       <c r="G80" t="n">
-        <v>4546.5</v>
+        <v>5357.86</v>
       </c>
       <c r="H80" t="inlineStr">
         <is>
@@ -4951,13 +4951,13 @@
         </is>
       </c>
       <c r="E81" t="n">
-        <v>3500</v>
+        <v>3623.39</v>
       </c>
       <c r="F81" t="n">
-        <v>288.75</v>
+        <v>298.93</v>
       </c>
       <c r="G81" t="n">
-        <v>3788.75</v>
+        <v>3922.32</v>
       </c>
       <c r="H81" t="inlineStr">
         <is>
@@ -4992,13 +4992,13 @@
         </is>
       </c>
       <c r="E82" t="n">
-        <v>1299</v>
+        <v>1057.02</v>
       </c>
       <c r="F82" t="n">
-        <v>107.17</v>
+        <v>87.20999999999999</v>
       </c>
       <c r="G82" t="n">
-        <v>1406.17</v>
+        <v>1144.23</v>
       </c>
       <c r="H82" t="inlineStr">
         <is>
@@ -5036,13 +5036,13 @@
         </is>
       </c>
       <c r="E83" t="n">
-        <v>699</v>
+        <v>568.79</v>
       </c>
       <c r="F83" t="n">
-        <v>57.67</v>
+        <v>46.93</v>
       </c>
       <c r="G83" t="n">
-        <v>756.67</v>
+        <v>615.72</v>
       </c>
       <c r="H83" t="inlineStr">
         <is>
@@ -5080,13 +5080,13 @@
         </is>
       </c>
       <c r="E84" t="n">
-        <v>2500</v>
+        <v>1869.95</v>
       </c>
       <c r="F84" t="n">
-        <v>206.25</v>
+        <v>154.27</v>
       </c>
       <c r="G84" t="n">
-        <v>2706.25</v>
+        <v>2024.22</v>
       </c>
       <c r="H84" t="inlineStr">
         <is>
@@ -5124,13 +5124,13 @@
         </is>
       </c>
       <c r="E85" t="n">
-        <v>1800</v>
+        <v>987.33</v>
       </c>
       <c r="F85" t="n">
-        <v>148.5</v>
+        <v>81.45</v>
       </c>
       <c r="G85" t="n">
-        <v>1948.5</v>
+        <v>1068.79</v>
       </c>
       <c r="H85" t="inlineStr">
         <is>
@@ -5165,13 +5165,13 @@
         </is>
       </c>
       <c r="E86" t="n">
-        <v>3500</v>
+        <v>2617.92</v>
       </c>
       <c r="F86" t="n">
-        <v>288.75</v>
+        <v>215.98</v>
       </c>
       <c r="G86" t="n">
-        <v>3788.75</v>
+        <v>2833.9</v>
       </c>
       <c r="H86" t="inlineStr">
         <is>
@@ -5209,13 +5209,13 @@
         </is>
       </c>
       <c r="E87" t="n">
-        <v>4200</v>
+        <v>3141.51</v>
       </c>
       <c r="F87" t="n">
-        <v>346.5</v>
+        <v>259.17</v>
       </c>
       <c r="G87" t="n">
-        <v>4546.5</v>
+        <v>3400.68</v>
       </c>
       <c r="H87" t="inlineStr">
         <is>
@@ -5253,13 +5253,13 @@
         </is>
       </c>
       <c r="E88" t="n">
-        <v>1399</v>
+        <v>1046.42</v>
       </c>
       <c r="F88" t="n">
-        <v>115.42</v>
+        <v>86.33</v>
       </c>
       <c r="G88" t="n">
-        <v>1514.42</v>
+        <v>1132.75</v>
       </c>
       <c r="H88" t="inlineStr">
         <is>
@@ -5297,13 +5297,13 @@
         </is>
       </c>
       <c r="E89" t="n">
-        <v>1899</v>
+        <v>1420.41</v>
       </c>
       <c r="F89" t="n">
-        <v>156.67</v>
+        <v>117.19</v>
       </c>
       <c r="G89" t="n">
-        <v>2055.67</v>
+        <v>1537.6</v>
       </c>
       <c r="H89" t="inlineStr">
         <is>
@@ -5338,13 +5338,13 @@
         </is>
       </c>
       <c r="E90" t="n">
-        <v>5500</v>
+        <v>4113.88</v>
       </c>
       <c r="F90" t="n">
-        <v>453.75</v>
+        <v>339.4</v>
       </c>
       <c r="G90" t="n">
-        <v>5953.75</v>
+        <v>4453.28</v>
       </c>
       <c r="H90" t="inlineStr">
         <is>
@@ -5382,13 +5382,13 @@
         </is>
       </c>
       <c r="E91" t="n">
-        <v>599</v>
+        <v>448.04</v>
       </c>
       <c r="F91" t="n">
-        <v>49.42</v>
+        <v>36.97</v>
       </c>
       <c r="G91" t="n">
-        <v>648.42</v>
+        <v>485</v>
       </c>
       <c r="H91" t="inlineStr">
         <is>
@@ -5489,13 +5489,13 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>8990</v>
+        <v>5170.71</v>
       </c>
       <c r="F2" t="n">
-        <v>741.6799999999999</v>
+        <v>426.59</v>
       </c>
       <c r="G2" t="n">
-        <v>9731.68</v>
+        <v>5597.3</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -5533,13 +5533,13 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>5592</v>
+        <v>3216.31</v>
       </c>
       <c r="F3" t="n">
-        <v>461.34</v>
+        <v>265.35</v>
       </c>
       <c r="G3" t="n">
-        <v>6053.34</v>
+        <v>3481.66</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -5577,13 +5577,13 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>3490</v>
+        <v>2007.32</v>
       </c>
       <c r="F4" t="n">
-        <v>287.93</v>
+        <v>165.61</v>
       </c>
       <c r="G4" t="n">
-        <v>3777.93</v>
+        <v>2172.92</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -5618,13 +5618,13 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>5094</v>
+        <v>7163.96</v>
       </c>
       <c r="F5" t="n">
-        <v>420.26</v>
+        <v>591.03</v>
       </c>
       <c r="G5" t="n">
-        <v>5514.26</v>
+        <v>7754.99</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -5662,13 +5662,13 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>3585</v>
+        <v>5041.77</v>
       </c>
       <c r="F6" t="n">
-        <v>295.76</v>
+        <v>415.94</v>
       </c>
       <c r="G6" t="n">
-        <v>3880.76</v>
+        <v>5457.72</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -5706,13 +5706,13 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>1788</v>
+        <v>3152.35</v>
       </c>
       <c r="F7" t="n">
-        <v>147.51</v>
+        <v>260.07</v>
       </c>
       <c r="G7" t="n">
-        <v>1935.51</v>
+        <v>3412.42</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -5750,13 +5750,13 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>7996</v>
+        <v>4896.82</v>
       </c>
       <c r="F8" t="n">
-        <v>659.67</v>
+        <v>403.99</v>
       </c>
       <c r="G8" t="n">
-        <v>8655.67</v>
+        <v>5300.8</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -5791,13 +5791,13 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>6060</v>
+        <v>3711.19</v>
       </c>
       <c r="F9" t="n">
-        <v>499.95</v>
+        <v>306.17</v>
       </c>
       <c r="G9" t="n">
-        <v>6559.95</v>
+        <v>4017.37</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -5832,13 +5832,13 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>6745</v>
+        <v>7542.7</v>
       </c>
       <c r="F10" t="n">
-        <v>556.46</v>
+        <v>622.27</v>
       </c>
       <c r="G10" t="n">
-        <v>7301.46</v>
+        <v>8164.97</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -5876,13 +5876,13 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>2475</v>
+        <v>4754.44</v>
       </c>
       <c r="F11" t="n">
-        <v>204.19</v>
+        <v>392.25</v>
       </c>
       <c r="G11" t="n">
-        <v>2679.19</v>
+        <v>5146.69</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -5917,13 +5917,13 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>7192</v>
+        <v>6006.53</v>
       </c>
       <c r="F12" t="n">
-        <v>593.34</v>
+        <v>495.54</v>
       </c>
       <c r="G12" t="n">
-        <v>7785.34</v>
+        <v>6502.07</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -5961,13 +5961,13 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>4194</v>
+        <v>4690.1</v>
       </c>
       <c r="F13" t="n">
-        <v>346.01</v>
+        <v>386.94</v>
       </c>
       <c r="G13" t="n">
-        <v>4540.01</v>
+        <v>5077.03</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -6002,13 +6002,13 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>2235</v>
+        <v>3528.75</v>
       </c>
       <c r="F14" t="n">
-        <v>184.39</v>
+        <v>291.13</v>
       </c>
       <c r="G14" t="n">
-        <v>2419.39</v>
+        <v>3819.88</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -6043,13 +6043,13 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>5394</v>
+        <v>7560.99</v>
       </c>
       <c r="F15" t="n">
-        <v>445.01</v>
+        <v>623.79</v>
       </c>
       <c r="G15" t="n">
-        <v>5839.01</v>
+        <v>8184.78</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -6084,13 +6084,13 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>5396</v>
+        <v>8495.030000000001</v>
       </c>
       <c r="F16" t="n">
-        <v>445.17</v>
+        <v>700.84</v>
       </c>
       <c r="G16" t="n">
-        <v>5841.17</v>
+        <v>9195.870000000001</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -6128,13 +6128,13 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>5997</v>
+        <v>3457.48</v>
       </c>
       <c r="F17" t="n">
-        <v>494.75</v>
+        <v>285.24</v>
       </c>
       <c r="G17" t="n">
-        <v>6491.75</v>
+        <v>3742.72</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -6169,13 +6169,13 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>5280</v>
+        <v>3036.86</v>
       </c>
       <c r="F18" t="n">
-        <v>435.6</v>
+        <v>250.54</v>
       </c>
       <c r="G18" t="n">
-        <v>5715.6</v>
+        <v>3287.4</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -6213,13 +6213,13 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>4790.4</v>
+        <v>8445.77</v>
       </c>
       <c r="F19" t="n">
-        <v>395.21</v>
+        <v>696.78</v>
       </c>
       <c r="G19" t="n">
-        <v>5185.61</v>
+        <v>9142.540000000001</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -6257,13 +6257,13 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>645</v>
+        <v>907.1</v>
       </c>
       <c r="F20" t="n">
-        <v>53.21</v>
+        <v>74.83</v>
       </c>
       <c r="G20" t="n">
-        <v>698.21</v>
+        <v>981.9299999999999</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -6301,13 +6301,13 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>525</v>
+        <v>587.09</v>
       </c>
       <c r="F21" t="n">
-        <v>43.31</v>
+        <v>48.43</v>
       </c>
       <c r="G21" t="n">
-        <v>568.3099999999999</v>
+        <v>635.52</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -6345,13 +6345,13 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>485</v>
+        <v>542.37</v>
       </c>
       <c r="F22" t="n">
-        <v>40.01</v>
+        <v>44.74</v>
       </c>
       <c r="G22" t="n">
-        <v>525.01</v>
+        <v>587.11</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -6389,13 +6389,13 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>565</v>
+        <v>889.49</v>
       </c>
       <c r="F23" t="n">
-        <v>46.61</v>
+        <v>73.38</v>
       </c>
       <c r="G23" t="n">
-        <v>611.61</v>
+        <v>962.87</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -6433,13 +6433,13 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>1800</v>
+        <v>1102.34</v>
       </c>
       <c r="F24" t="n">
-        <v>148.5</v>
+        <v>90.94</v>
       </c>
       <c r="G24" t="n">
-        <v>1948.5</v>
+        <v>1193.28</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
@@ -6474,13 +6474,13 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>1600</v>
+        <v>2526.18</v>
       </c>
       <c r="F25" t="n">
-        <v>132</v>
+        <v>208.41</v>
       </c>
       <c r="G25" t="n">
-        <v>1732</v>
+        <v>2734.59</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
@@ -6518,13 +6518,13 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>1200</v>
+        <v>2305.18</v>
       </c>
       <c r="F26" t="n">
-        <v>99</v>
+        <v>190.18</v>
       </c>
       <c r="G26" t="n">
-        <v>1299</v>
+        <v>2495.36</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
@@ -6559,13 +6559,13 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>45</v>
+        <v>25.94</v>
       </c>
       <c r="F27" t="n">
-        <v>3.71</v>
+        <v>2.14</v>
       </c>
       <c r="G27" t="n">
-        <v>48.71</v>
+        <v>28.08</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
@@ -6603,13 +6603,13 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>8990</v>
+        <v>5183.04</v>
       </c>
       <c r="F28" t="n">
-        <v>741.6799999999999</v>
+        <v>427.6</v>
       </c>
       <c r="G28" t="n">
-        <v>9731.68</v>
+        <v>5610.65</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
@@ -6647,13 +6647,13 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>32</v>
+        <v>18.45</v>
       </c>
       <c r="F29" t="n">
-        <v>2.64</v>
+        <v>1.52</v>
       </c>
       <c r="G29" t="n">
-        <v>34.64</v>
+        <v>19.97</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
@@ -6691,13 +6691,13 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>3490</v>
+        <v>2012.1</v>
       </c>
       <c r="F30" t="n">
-        <v>287.93</v>
+        <v>166</v>
       </c>
       <c r="G30" t="n">
-        <v>3777.93</v>
+        <v>2178.11</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
@@ -6735,13 +6735,13 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>565</v>
+        <v>325.74</v>
       </c>
       <c r="F31" t="n">
-        <v>46.61</v>
+        <v>26.87</v>
       </c>
       <c r="G31" t="n">
-        <v>611.61</v>
+        <v>352.61</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
@@ -6779,13 +6779,13 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>3600</v>
+        <v>3252.75</v>
       </c>
       <c r="F32" t="n">
-        <v>297</v>
+        <v>268.35</v>
       </c>
       <c r="G32" t="n">
-        <v>3897</v>
+        <v>3521.1</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
@@ -6820,13 +6820,13 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>1680</v>
+        <v>1517.95</v>
       </c>
       <c r="F33" t="n">
-        <v>138.6</v>
+        <v>125.23</v>
       </c>
       <c r="G33" t="n">
-        <v>1818.6</v>
+        <v>1643.18</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
@@ -6861,13 +6861,13 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>1140</v>
+        <v>1030.04</v>
       </c>
       <c r="F34" t="n">
-        <v>94.05</v>
+        <v>84.98</v>
       </c>
       <c r="G34" t="n">
-        <v>1234.05</v>
+        <v>1115.02</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
@@ -6902,13 +6902,13 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>4245</v>
+        <v>3835.53</v>
       </c>
       <c r="F35" t="n">
-        <v>350.21</v>
+        <v>316.43</v>
       </c>
       <c r="G35" t="n">
-        <v>4595.21</v>
+        <v>4151.96</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
@@ -6943,13 +6943,13 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>2392</v>
+        <v>2161.27</v>
       </c>
       <c r="F36" t="n">
-        <v>197.34</v>
+        <v>178.3</v>
       </c>
       <c r="G36" t="n">
-        <v>2589.34</v>
+        <v>2339.58</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>

</xml_diff>